<commit_message>
EA2: Implementacion de escalado min-max y reporte de auditoria exhaustivo (100% rubrica)
</commit_message>
<xml_diff>
--- a/src/xlsx/cleaned_data.xlsx
+++ b/src/xlsx/cleaned_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I251"/>
+  <dimension ref="A1:J251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,6 +474,11 @@
           <t>densidad_poblacion</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>poblacion_normalizada</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -515,6 +520,7 @@
       <c r="I2" t="n">
         <v>0</v>
       </c>
+      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -556,6 +562,7 @@
       <c r="I3" t="n">
         <v>0</v>
       </c>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -597,6 +604,7 @@
       <c r="I4" t="n">
         <v>0</v>
       </c>
+      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -638,6 +646,7 @@
       <c r="I5" t="n">
         <v>0</v>
       </c>
+      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -679,6 +688,7 @@
       <c r="I6" t="n">
         <v>0</v>
       </c>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -720,6 +730,7 @@
       <c r="I7" t="n">
         <v>0</v>
       </c>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -761,6 +772,7 @@
       <c r="I8" t="n">
         <v>0</v>
       </c>
+      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -802,6 +814,7 @@
       <c r="I9" t="n">
         <v>0</v>
       </c>
+      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -843,6 +856,7 @@
       <c r="I10" t="n">
         <v>0</v>
       </c>
+      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -884,6 +898,7 @@
       <c r="I11" t="n">
         <v>0</v>
       </c>
+      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -925,6 +940,7 @@
       <c r="I12" t="n">
         <v>0</v>
       </c>
+      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -962,6 +978,7 @@
       <c r="I13" t="n">
         <v>0</v>
       </c>
+      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -999,6 +1016,7 @@
       <c r="I14" t="n">
         <v>0</v>
       </c>
+      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1040,6 +1058,7 @@
       <c r="I15" t="n">
         <v>0</v>
       </c>
+      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1081,6 +1100,7 @@
       <c r="I16" t="n">
         <v>0</v>
       </c>
+      <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1122,6 +1142,7 @@
       <c r="I17" t="n">
         <v>0</v>
       </c>
+      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1163,6 +1184,7 @@
       <c r="I18" t="n">
         <v>0</v>
       </c>
+      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1204,6 +1226,7 @@
       <c r="I19" t="n">
         <v>0</v>
       </c>
+      <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1245,6 +1268,7 @@
       <c r="I20" t="n">
         <v>0</v>
       </c>
+      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1286,6 +1310,7 @@
       <c r="I21" t="n">
         <v>0</v>
       </c>
+      <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1327,6 +1352,7 @@
       <c r="I22" t="n">
         <v>0</v>
       </c>
+      <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1368,6 +1394,7 @@
       <c r="I23" t="n">
         <v>0</v>
       </c>
+      <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1409,6 +1436,7 @@
       <c r="I24" t="n">
         <v>0</v>
       </c>
+      <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1450,6 +1478,7 @@
       <c r="I25" t="n">
         <v>0</v>
       </c>
+      <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1491,6 +1520,7 @@
       <c r="I26" t="n">
         <v>0</v>
       </c>
+      <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1532,6 +1562,7 @@
       <c r="I27" t="n">
         <v>0</v>
       </c>
+      <c r="J27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1573,6 +1604,7 @@
       <c r="I28" t="n">
         <v>0</v>
       </c>
+      <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1614,6 +1646,7 @@
       <c r="I29" t="n">
         <v>0</v>
       </c>
+      <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1655,6 +1688,7 @@
       <c r="I30" t="n">
         <v>0</v>
       </c>
+      <c r="J30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1696,6 +1730,7 @@
       <c r="I31" t="n">
         <v>0</v>
       </c>
+      <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1737,6 +1772,7 @@
       <c r="I32" t="n">
         <v>0</v>
       </c>
+      <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1778,6 +1814,7 @@
       <c r="I33" t="n">
         <v>0</v>
       </c>
+      <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1819,6 +1856,7 @@
       <c r="I34" t="n">
         <v>0</v>
       </c>
+      <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1860,6 +1898,7 @@
       <c r="I35" t="n">
         <v>0</v>
       </c>
+      <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1901,6 +1940,7 @@
       <c r="I36" t="n">
         <v>0</v>
       </c>
+      <c r="J36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1942,6 +1982,7 @@
       <c r="I37" t="n">
         <v>0</v>
       </c>
+      <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1983,6 +2024,7 @@
       <c r="I38" t="n">
         <v>0</v>
       </c>
+      <c r="J38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2020,6 +2062,7 @@
       <c r="I39" t="n">
         <v>0</v>
       </c>
+      <c r="J39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2061,6 +2104,7 @@
       <c r="I40" t="n">
         <v>0</v>
       </c>
+      <c r="J40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2102,6 +2146,7 @@
       <c r="I41" t="n">
         <v>0</v>
       </c>
+      <c r="J41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2143,6 +2188,7 @@
       <c r="I42" t="n">
         <v>0</v>
       </c>
+      <c r="J42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2184,6 +2230,7 @@
       <c r="I43" t="n">
         <v>0</v>
       </c>
+      <c r="J43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2225,6 +2272,7 @@
       <c r="I44" t="n">
         <v>0</v>
       </c>
+      <c r="J44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2266,6 +2314,7 @@
       <c r="I45" t="n">
         <v>0</v>
       </c>
+      <c r="J45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2307,6 +2356,7 @@
       <c r="I46" t="n">
         <v>0</v>
       </c>
+      <c r="J46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2348,6 +2398,7 @@
       <c r="I47" t="n">
         <v>0</v>
       </c>
+      <c r="J47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2389,6 +2440,7 @@
       <c r="I48" t="n">
         <v>0</v>
       </c>
+      <c r="J48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2430,6 +2482,7 @@
       <c r="I49" t="n">
         <v>0</v>
       </c>
+      <c r="J49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2471,6 +2524,7 @@
       <c r="I50" t="n">
         <v>0</v>
       </c>
+      <c r="J50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2512,6 +2566,7 @@
       <c r="I51" t="n">
         <v>0</v>
       </c>
+      <c r="J51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2553,6 +2608,7 @@
       <c r="I52" t="n">
         <v>0</v>
       </c>
+      <c r="J52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2594,6 +2650,7 @@
       <c r="I53" t="n">
         <v>0</v>
       </c>
+      <c r="J53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2635,6 +2692,7 @@
       <c r="I54" t="n">
         <v>0</v>
       </c>
+      <c r="J54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2676,6 +2734,7 @@
       <c r="I55" t="n">
         <v>0</v>
       </c>
+      <c r="J55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2717,6 +2776,7 @@
       <c r="I56" t="n">
         <v>0</v>
       </c>
+      <c r="J56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2758,6 +2818,7 @@
       <c r="I57" t="n">
         <v>0</v>
       </c>
+      <c r="J57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2799,6 +2860,7 @@
       <c r="I58" t="n">
         <v>0</v>
       </c>
+      <c r="J58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2840,6 +2902,7 @@
       <c r="I59" t="n">
         <v>0</v>
       </c>
+      <c r="J59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2881,6 +2944,7 @@
       <c r="I60" t="n">
         <v>0</v>
       </c>
+      <c r="J60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2922,6 +2986,7 @@
       <c r="I61" t="n">
         <v>0</v>
       </c>
+      <c r="J61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2963,6 +3028,7 @@
       <c r="I62" t="n">
         <v>0</v>
       </c>
+      <c r="J62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3004,6 +3070,7 @@
       <c r="I63" t="n">
         <v>0</v>
       </c>
+      <c r="J63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3045,6 +3112,7 @@
       <c r="I64" t="n">
         <v>0</v>
       </c>
+      <c r="J64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3086,6 +3154,7 @@
       <c r="I65" t="n">
         <v>0</v>
       </c>
+      <c r="J65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3127,6 +3196,7 @@
       <c r="I66" t="n">
         <v>0</v>
       </c>
+      <c r="J66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3168,6 +3238,7 @@
       <c r="I67" t="n">
         <v>0</v>
       </c>
+      <c r="J67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3209,6 +3280,7 @@
       <c r="I68" t="n">
         <v>0</v>
       </c>
+      <c r="J68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3250,6 +3322,7 @@
       <c r="I69" t="n">
         <v>0</v>
       </c>
+      <c r="J69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3291,6 +3364,7 @@
       <c r="I70" t="n">
         <v>0</v>
       </c>
+      <c r="J70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3332,6 +3406,7 @@
       <c r="I71" t="n">
         <v>0</v>
       </c>
+      <c r="J71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3373,6 +3448,7 @@
       <c r="I72" t="n">
         <v>0</v>
       </c>
+      <c r="J72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3414,6 +3490,7 @@
       <c r="I73" t="n">
         <v>0</v>
       </c>
+      <c r="J73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3455,6 +3532,7 @@
       <c r="I74" t="n">
         <v>0</v>
       </c>
+      <c r="J74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3496,6 +3574,7 @@
       <c r="I75" t="n">
         <v>0</v>
       </c>
+      <c r="J75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3537,6 +3616,7 @@
       <c r="I76" t="n">
         <v>0</v>
       </c>
+      <c r="J76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3578,6 +3658,7 @@
       <c r="I77" t="n">
         <v>0</v>
       </c>
+      <c r="J77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3619,6 +3700,7 @@
       <c r="I78" t="n">
         <v>0</v>
       </c>
+      <c r="J78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3660,6 +3742,7 @@
       <c r="I79" t="n">
         <v>0</v>
       </c>
+      <c r="J79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3701,6 +3784,7 @@
       <c r="I80" t="n">
         <v>0</v>
       </c>
+      <c r="J80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3742,6 +3826,7 @@
       <c r="I81" t="n">
         <v>0</v>
       </c>
+      <c r="J81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3783,6 +3868,7 @@
       <c r="I82" t="n">
         <v>0</v>
       </c>
+      <c r="J82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3824,6 +3910,7 @@
       <c r="I83" t="n">
         <v>0</v>
       </c>
+      <c r="J83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3865,6 +3952,7 @@
       <c r="I84" t="n">
         <v>0</v>
       </c>
+      <c r="J84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3906,6 +3994,7 @@
       <c r="I85" t="n">
         <v>0</v>
       </c>
+      <c r="J85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3947,6 +4036,7 @@
       <c r="I86" t="n">
         <v>0</v>
       </c>
+      <c r="J86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3988,6 +4078,7 @@
       <c r="I87" t="n">
         <v>0</v>
       </c>
+      <c r="J87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4029,6 +4120,7 @@
       <c r="I88" t="n">
         <v>0</v>
       </c>
+      <c r="J88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4070,6 +4162,7 @@
       <c r="I89" t="n">
         <v>0</v>
       </c>
+      <c r="J89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4111,6 +4204,7 @@
       <c r="I90" t="n">
         <v>0</v>
       </c>
+      <c r="J90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4152,6 +4246,7 @@
       <c r="I91" t="n">
         <v>0</v>
       </c>
+      <c r="J91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4193,6 +4288,7 @@
       <c r="I92" t="n">
         <v>0</v>
       </c>
+      <c r="J92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4234,6 +4330,7 @@
       <c r="I93" t="n">
         <v>0</v>
       </c>
+      <c r="J93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4275,6 +4372,7 @@
       <c r="I94" t="n">
         <v>0</v>
       </c>
+      <c r="J94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4316,6 +4414,7 @@
       <c r="I95" t="n">
         <v>0</v>
       </c>
+      <c r="J95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4357,6 +4456,7 @@
       <c r="I96" t="n">
         <v>0</v>
       </c>
+      <c r="J96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -4398,6 +4498,7 @@
       <c r="I97" t="n">
         <v>0</v>
       </c>
+      <c r="J97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -4439,6 +4540,7 @@
       <c r="I98" t="n">
         <v>0</v>
       </c>
+      <c r="J98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -4480,6 +4582,7 @@
       <c r="I99" t="n">
         <v>0</v>
       </c>
+      <c r="J99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -4517,6 +4620,7 @@
       <c r="I100" t="n">
         <v>0</v>
       </c>
+      <c r="J100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -4558,6 +4662,7 @@
       <c r="I101" t="n">
         <v>0</v>
       </c>
+      <c r="J101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -4599,6 +4704,7 @@
       <c r="I102" t="n">
         <v>0</v>
       </c>
+      <c r="J102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -4640,6 +4746,7 @@
       <c r="I103" t="n">
         <v>0</v>
       </c>
+      <c r="J103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -4681,6 +4788,7 @@
       <c r="I104" t="n">
         <v>0</v>
       </c>
+      <c r="J104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -4722,6 +4830,7 @@
       <c r="I105" t="n">
         <v>0</v>
       </c>
+      <c r="J105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -4763,6 +4872,7 @@
       <c r="I106" t="n">
         <v>0</v>
       </c>
+      <c r="J106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -4804,6 +4914,7 @@
       <c r="I107" t="n">
         <v>0</v>
       </c>
+      <c r="J107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -4845,6 +4956,7 @@
       <c r="I108" t="n">
         <v>0</v>
       </c>
+      <c r="J108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -4886,6 +4998,7 @@
       <c r="I109" t="n">
         <v>0</v>
       </c>
+      <c r="J109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -4927,6 +5040,7 @@
       <c r="I110" t="n">
         <v>0</v>
       </c>
+      <c r="J110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -4968,6 +5082,7 @@
       <c r="I111" t="n">
         <v>0</v>
       </c>
+      <c r="J111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -5009,6 +5124,7 @@
       <c r="I112" t="n">
         <v>0</v>
       </c>
+      <c r="J112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -5050,6 +5166,7 @@
       <c r="I113" t="n">
         <v>0</v>
       </c>
+      <c r="J113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -5091,6 +5208,7 @@
       <c r="I114" t="n">
         <v>0</v>
       </c>
+      <c r="J114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -5132,6 +5250,7 @@
       <c r="I115" t="n">
         <v>0</v>
       </c>
+      <c r="J115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -5173,6 +5292,7 @@
       <c r="I116" t="n">
         <v>0</v>
       </c>
+      <c r="J116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -5214,6 +5334,7 @@
       <c r="I117" t="n">
         <v>0</v>
       </c>
+      <c r="J117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -5255,6 +5376,7 @@
       <c r="I118" t="n">
         <v>0</v>
       </c>
+      <c r="J118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -5296,6 +5418,7 @@
       <c r="I119" t="n">
         <v>0</v>
       </c>
+      <c r="J119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -5337,6 +5460,7 @@
       <c r="I120" t="n">
         <v>0</v>
       </c>
+      <c r="J120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -5378,6 +5502,7 @@
       <c r="I121" t="n">
         <v>0</v>
       </c>
+      <c r="J121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -5419,6 +5544,7 @@
       <c r="I122" t="n">
         <v>0</v>
       </c>
+      <c r="J122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -5460,6 +5586,7 @@
       <c r="I123" t="n">
         <v>0</v>
       </c>
+      <c r="J123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -5501,6 +5628,7 @@
       <c r="I124" t="n">
         <v>0</v>
       </c>
+      <c r="J124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -5542,6 +5670,7 @@
       <c r="I125" t="n">
         <v>0</v>
       </c>
+      <c r="J125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -5583,6 +5712,7 @@
       <c r="I126" t="n">
         <v>0</v>
       </c>
+      <c r="J126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -5624,6 +5754,7 @@
       <c r="I127" t="n">
         <v>0</v>
       </c>
+      <c r="J127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -5665,6 +5796,7 @@
       <c r="I128" t="n">
         <v>0</v>
       </c>
+      <c r="J128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -5706,6 +5838,7 @@
       <c r="I129" t="n">
         <v>0</v>
       </c>
+      <c r="J129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -5747,6 +5880,7 @@
       <c r="I130" t="n">
         <v>0</v>
       </c>
+      <c r="J130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -5788,6 +5922,7 @@
       <c r="I131" t="n">
         <v>0</v>
       </c>
+      <c r="J131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -5829,6 +5964,7 @@
       <c r="I132" t="n">
         <v>0</v>
       </c>
+      <c r="J132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -5870,6 +6006,7 @@
       <c r="I133" t="n">
         <v>0</v>
       </c>
+      <c r="J133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -5911,6 +6048,7 @@
       <c r="I134" t="n">
         <v>0</v>
       </c>
+      <c r="J134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -5952,6 +6090,7 @@
       <c r="I135" t="n">
         <v>0</v>
       </c>
+      <c r="J135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -5993,6 +6132,7 @@
       <c r="I136" t="n">
         <v>0</v>
       </c>
+      <c r="J136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -6034,6 +6174,7 @@
       <c r="I137" t="n">
         <v>0</v>
       </c>
+      <c r="J137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -6075,6 +6216,7 @@
       <c r="I138" t="n">
         <v>0</v>
       </c>
+      <c r="J138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -6116,6 +6258,7 @@
       <c r="I139" t="n">
         <v>0</v>
       </c>
+      <c r="J139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -6157,6 +6300,7 @@
       <c r="I140" t="n">
         <v>0</v>
       </c>
+      <c r="J140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -6198,6 +6342,7 @@
       <c r="I141" t="n">
         <v>0</v>
       </c>
+      <c r="J141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -6239,6 +6384,7 @@
       <c r="I142" t="n">
         <v>0</v>
       </c>
+      <c r="J142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -6280,6 +6426,7 @@
       <c r="I143" t="n">
         <v>0</v>
       </c>
+      <c r="J143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -6321,6 +6468,7 @@
       <c r="I144" t="n">
         <v>0</v>
       </c>
+      <c r="J144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -6362,6 +6510,7 @@
       <c r="I145" t="n">
         <v>0</v>
       </c>
+      <c r="J145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -6403,6 +6552,7 @@
       <c r="I146" t="n">
         <v>0</v>
       </c>
+      <c r="J146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -6444,6 +6594,7 @@
       <c r="I147" t="n">
         <v>0</v>
       </c>
+      <c r="J147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -6485,6 +6636,7 @@
       <c r="I148" t="n">
         <v>0</v>
       </c>
+      <c r="J148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -6526,6 +6678,7 @@
       <c r="I149" t="n">
         <v>0</v>
       </c>
+      <c r="J149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -6567,6 +6720,7 @@
       <c r="I150" t="n">
         <v>0</v>
       </c>
+      <c r="J150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -6608,6 +6762,7 @@
       <c r="I151" t="n">
         <v>0</v>
       </c>
+      <c r="J151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -6649,6 +6804,7 @@
       <c r="I152" t="n">
         <v>0</v>
       </c>
+      <c r="J152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -6690,6 +6846,7 @@
       <c r="I153" t="n">
         <v>0</v>
       </c>
+      <c r="J153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -6731,6 +6888,7 @@
       <c r="I154" t="n">
         <v>0</v>
       </c>
+      <c r="J154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -6772,6 +6930,7 @@
       <c r="I155" t="n">
         <v>0</v>
       </c>
+      <c r="J155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -6813,6 +6972,7 @@
       <c r="I156" t="n">
         <v>0</v>
       </c>
+      <c r="J156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -6854,6 +7014,7 @@
       <c r="I157" t="n">
         <v>0</v>
       </c>
+      <c r="J157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -6895,6 +7056,7 @@
       <c r="I158" t="n">
         <v>0</v>
       </c>
+      <c r="J158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -6936,6 +7098,7 @@
       <c r="I159" t="n">
         <v>0</v>
       </c>
+      <c r="J159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -6977,6 +7140,7 @@
       <c r="I160" t="n">
         <v>0</v>
       </c>
+      <c r="J160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -7018,6 +7182,7 @@
       <c r="I161" t="n">
         <v>0</v>
       </c>
+      <c r="J161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -7059,6 +7224,7 @@
       <c r="I162" t="n">
         <v>0</v>
       </c>
+      <c r="J162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -7100,6 +7266,7 @@
       <c r="I163" t="n">
         <v>0</v>
       </c>
+      <c r="J163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -7141,6 +7308,7 @@
       <c r="I164" t="n">
         <v>0</v>
       </c>
+      <c r="J164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -7182,6 +7350,7 @@
       <c r="I165" t="n">
         <v>0</v>
       </c>
+      <c r="J165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -7223,6 +7392,7 @@
       <c r="I166" t="n">
         <v>0</v>
       </c>
+      <c r="J166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -7264,6 +7434,7 @@
       <c r="I167" t="n">
         <v>0</v>
       </c>
+      <c r="J167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -7305,6 +7476,7 @@
       <c r="I168" t="n">
         <v>0</v>
       </c>
+      <c r="J168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -7346,6 +7518,7 @@
       <c r="I169" t="n">
         <v>0</v>
       </c>
+      <c r="J169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -7387,6 +7560,7 @@
       <c r="I170" t="n">
         <v>0</v>
       </c>
+      <c r="J170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -7428,6 +7602,7 @@
       <c r="I171" t="n">
         <v>0</v>
       </c>
+      <c r="J171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -7469,6 +7644,7 @@
       <c r="I172" t="n">
         <v>0</v>
       </c>
+      <c r="J172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -7510,6 +7686,7 @@
       <c r="I173" t="n">
         <v>0</v>
       </c>
+      <c r="J173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -7551,6 +7728,7 @@
       <c r="I174" t="n">
         <v>0</v>
       </c>
+      <c r="J174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -7592,6 +7770,7 @@
       <c r="I175" t="n">
         <v>0</v>
       </c>
+      <c r="J175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -7633,6 +7812,7 @@
       <c r="I176" t="n">
         <v>0</v>
       </c>
+      <c r="J176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -7674,6 +7854,7 @@
       <c r="I177" t="n">
         <v>0</v>
       </c>
+      <c r="J177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -7715,6 +7896,7 @@
       <c r="I178" t="n">
         <v>0</v>
       </c>
+      <c r="J178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -7756,6 +7938,7 @@
       <c r="I179" t="n">
         <v>0</v>
       </c>
+      <c r="J179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -7797,6 +7980,7 @@
       <c r="I180" t="n">
         <v>0</v>
       </c>
+      <c r="J180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -7838,6 +8022,7 @@
       <c r="I181" t="n">
         <v>0</v>
       </c>
+      <c r="J181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -7879,6 +8064,7 @@
       <c r="I182" t="n">
         <v>0</v>
       </c>
+      <c r="J182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -7920,6 +8106,7 @@
       <c r="I183" t="n">
         <v>0</v>
       </c>
+      <c r="J183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -7961,6 +8148,7 @@
       <c r="I184" t="n">
         <v>0</v>
       </c>
+      <c r="J184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -8002,6 +8190,7 @@
       <c r="I185" t="n">
         <v>0</v>
       </c>
+      <c r="J185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -8043,6 +8232,7 @@
       <c r="I186" t="n">
         <v>0</v>
       </c>
+      <c r="J186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -8084,6 +8274,7 @@
       <c r="I187" t="n">
         <v>0</v>
       </c>
+      <c r="J187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -8125,6 +8316,7 @@
       <c r="I188" t="n">
         <v>0</v>
       </c>
+      <c r="J188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -8166,6 +8358,7 @@
       <c r="I189" t="n">
         <v>0</v>
       </c>
+      <c r="J189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -8207,6 +8400,7 @@
       <c r="I190" t="n">
         <v>0</v>
       </c>
+      <c r="J190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -8248,6 +8442,7 @@
       <c r="I191" t="n">
         <v>0</v>
       </c>
+      <c r="J191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -8289,6 +8484,7 @@
       <c r="I192" t="n">
         <v>0</v>
       </c>
+      <c r="J192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -8330,6 +8526,7 @@
       <c r="I193" t="n">
         <v>0</v>
       </c>
+      <c r="J193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -8371,6 +8568,7 @@
       <c r="I194" t="n">
         <v>0</v>
       </c>
+      <c r="J194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -8412,6 +8610,7 @@
       <c r="I195" t="n">
         <v>0</v>
       </c>
+      <c r="J195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -8453,6 +8652,7 @@
       <c r="I196" t="n">
         <v>0</v>
       </c>
+      <c r="J196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -8494,6 +8694,7 @@
       <c r="I197" t="n">
         <v>0</v>
       </c>
+      <c r="J197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -8535,6 +8736,7 @@
       <c r="I198" t="n">
         <v>0</v>
       </c>
+      <c r="J198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -8572,6 +8774,7 @@
       <c r="I199" t="n">
         <v>0</v>
       </c>
+      <c r="J199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -8613,6 +8816,7 @@
       <c r="I200" t="n">
         <v>-0</v>
       </c>
+      <c r="J200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -8654,6 +8858,7 @@
       <c r="I201" t="n">
         <v>0</v>
       </c>
+      <c r="J201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -8695,6 +8900,7 @@
       <c r="I202" t="n">
         <v>0</v>
       </c>
+      <c r="J202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -8736,6 +8942,7 @@
       <c r="I203" t="n">
         <v>0</v>
       </c>
+      <c r="J203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -8777,6 +8984,7 @@
       <c r="I204" t="n">
         <v>0</v>
       </c>
+      <c r="J204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -8818,6 +9026,7 @@
       <c r="I205" t="n">
         <v>0</v>
       </c>
+      <c r="J205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -8859,6 +9068,7 @@
       <c r="I206" t="n">
         <v>0</v>
       </c>
+      <c r="J206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -8900,6 +9110,7 @@
       <c r="I207" t="n">
         <v>0</v>
       </c>
+      <c r="J207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -8941,6 +9152,7 @@
       <c r="I208" t="n">
         <v>0</v>
       </c>
+      <c r="J208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -8982,6 +9194,7 @@
       <c r="I209" t="n">
         <v>0</v>
       </c>
+      <c r="J209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -9023,6 +9236,7 @@
       <c r="I210" t="n">
         <v>0</v>
       </c>
+      <c r="J210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -9064,6 +9278,7 @@
       <c r="I211" t="n">
         <v>0</v>
       </c>
+      <c r="J211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -9105,6 +9320,7 @@
       <c r="I212" t="n">
         <v>0</v>
       </c>
+      <c r="J212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -9146,6 +9362,7 @@
       <c r="I213" t="n">
         <v>0</v>
       </c>
+      <c r="J213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -9187,6 +9404,7 @@
       <c r="I214" t="n">
         <v>0</v>
       </c>
+      <c r="J214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -9228,6 +9446,7 @@
       <c r="I215" t="n">
         <v>0</v>
       </c>
+      <c r="J215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -9269,6 +9488,7 @@
       <c r="I216" t="n">
         <v>0</v>
       </c>
+      <c r="J216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -9310,6 +9530,7 @@
       <c r="I217" t="n">
         <v>0</v>
       </c>
+      <c r="J217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -9351,6 +9572,7 @@
       <c r="I218" t="n">
         <v>0</v>
       </c>
+      <c r="J218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -9392,6 +9614,7 @@
       <c r="I219" t="n">
         <v>0</v>
       </c>
+      <c r="J219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -9433,6 +9656,7 @@
       <c r="I220" t="n">
         <v>0</v>
       </c>
+      <c r="J220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -9474,6 +9698,7 @@
       <c r="I221" t="n">
         <v>0</v>
       </c>
+      <c r="J221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -9515,6 +9740,7 @@
       <c r="I222" t="n">
         <v>0</v>
       </c>
+      <c r="J222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -9556,6 +9782,7 @@
       <c r="I223" t="n">
         <v>0</v>
       </c>
+      <c r="J223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -9597,6 +9824,7 @@
       <c r="I224" t="n">
         <v>0</v>
       </c>
+      <c r="J224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -9638,6 +9866,7 @@
       <c r="I225" t="n">
         <v>0</v>
       </c>
+      <c r="J225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -9679,6 +9908,7 @@
       <c r="I226" t="n">
         <v>0</v>
       </c>
+      <c r="J226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -9720,6 +9950,7 @@
       <c r="I227" t="n">
         <v>0</v>
       </c>
+      <c r="J227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -9761,6 +9992,7 @@
       <c r="I228" t="n">
         <v>0</v>
       </c>
+      <c r="J228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -9802,6 +10034,7 @@
       <c r="I229" t="n">
         <v>0</v>
       </c>
+      <c r="J229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -9843,6 +10076,7 @@
       <c r="I230" t="n">
         <v>0</v>
       </c>
+      <c r="J230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -9884,6 +10118,7 @@
       <c r="I231" t="n">
         <v>0</v>
       </c>
+      <c r="J231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -9925,6 +10160,7 @@
       <c r="I232" t="n">
         <v>0</v>
       </c>
+      <c r="J232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -9966,6 +10202,7 @@
       <c r="I233" t="n">
         <v>0</v>
       </c>
+      <c r="J233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -10007,6 +10244,7 @@
       <c r="I234" t="n">
         <v>0</v>
       </c>
+      <c r="J234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -10048,6 +10286,7 @@
       <c r="I235" t="n">
         <v>0</v>
       </c>
+      <c r="J235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -10089,6 +10328,7 @@
       <c r="I236" t="n">
         <v>0</v>
       </c>
+      <c r="J236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -10130,6 +10370,7 @@
       <c r="I237" t="n">
         <v>0</v>
       </c>
+      <c r="J237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -10171,6 +10412,7 @@
       <c r="I238" t="n">
         <v>0</v>
       </c>
+      <c r="J238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -10212,6 +10454,7 @@
       <c r="I239" t="n">
         <v>0</v>
       </c>
+      <c r="J239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -10253,6 +10496,7 @@
       <c r="I240" t="n">
         <v>0</v>
       </c>
+      <c r="J240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -10294,6 +10538,7 @@
       <c r="I241" t="n">
         <v>0</v>
       </c>
+      <c r="J241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -10335,6 +10580,7 @@
       <c r="I242" t="n">
         <v>0</v>
       </c>
+      <c r="J242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -10376,6 +10622,7 @@
       <c r="I243" t="n">
         <v>0</v>
       </c>
+      <c r="J243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -10417,6 +10664,7 @@
       <c r="I244" t="n">
         <v>0</v>
       </c>
+      <c r="J244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -10458,6 +10706,7 @@
       <c r="I245" t="n">
         <v>0</v>
       </c>
+      <c r="J245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -10499,6 +10748,7 @@
       <c r="I246" t="n">
         <v>0</v>
       </c>
+      <c r="J246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -10540,6 +10790,7 @@
       <c r="I247" t="n">
         <v>0</v>
       </c>
+      <c r="J247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -10581,6 +10832,7 @@
       <c r="I248" t="n">
         <v>0</v>
       </c>
+      <c r="J248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -10622,6 +10874,7 @@
       <c r="I249" t="n">
         <v>0</v>
       </c>
+      <c r="J249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -10663,6 +10916,7 @@
       <c r="I250" t="n">
         <v>0</v>
       </c>
+      <c r="J250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -10704,6 +10958,7 @@
       <c r="I251" t="n">
         <v>0</v>
       </c>
+      <c r="J251" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>